<commit_message>
fix(multi-conta): correcoes do QA gate da 7.3 [Story 7.3]
- QA-731-1: coluna conta_emissora nos modelos baixaveis (csv + xlsx regenerado)
- QA-731-2: teste de rota do 503 CONTA_NAO_CONFIGURADA (remediacao D-721 coberta)
- 295 testes verdes no total

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/medicos-modelo.xlsx
+++ b/apps/web/public/templates/medicos-modelo.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Médicos" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Medicos" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="56">
   <si>
     <t>cpf</t>
   </si>
@@ -46,9 +46,6 @@
     <t>pagador_nome</t>
   </si>
   <si>
-    <t>whatsapp</t>
-  </si>
-  <si>
     <t>email</t>
   </si>
   <si>
@@ -73,6 +70,9 @@
     <t>uf</t>
   </si>
   <si>
+    <t>conta_emissora</t>
+  </si>
+  <si>
     <t>12345678900</t>
   </si>
   <si>
@@ -94,9 +94,6 @@
     <t>PF</t>
   </si>
   <si>
-    <t>5511999999999</t>
-  </si>
-  <si>
     <t>fulano@exemplo.com</t>
   </si>
   <si>
@@ -121,6 +118,9 @@
     <t>CE</t>
   </si>
   <si>
+    <t>mc</t>
+  </si>
+  <si>
     <t>98765432100</t>
   </si>
   <si>
@@ -145,9 +145,6 @@
     <t>Clinica Ciclana LTDA</t>
   </si>
   <si>
-    <t>5511888888888</t>
-  </si>
-  <si>
     <t>contato@ciclana.com</t>
   </si>
   <si>
@@ -164,6 +161,24 @@
   </si>
   <si>
     <t>Meireles</t>
+  </si>
+  <si>
+    <t>cavalcante_viana</t>
+  </si>
+  <si>
+    <t>11122233344</t>
+  </si>
+  <si>
+    <t>Dr. Beltrano</t>
+  </si>
+  <si>
+    <t>Ortopedia</t>
+  </si>
+  <si>
+    <t>nenhum</t>
+  </si>
+  <si>
+    <t>sim</t>
   </si>
 </sst>
 </file>
@@ -180,20 +195,14 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F2937"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -210,9 +219,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -552,26 +559,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="7" width="20" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="7" width="19" customWidth="1"/>
     <col min="8" max="8" width="25" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
-    <col min="11" max="11" width="30" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
-    <col min="13" max="13" width="30" customWidth="1"/>
-    <col min="14" max="14" width="15" customWidth="1"/>
-    <col min="15" max="15" width="30" customWidth="1"/>
-    <col min="16" max="16" width="10" customWidth="1"/>
-    <col min="17" max="19" width="20" customWidth="1"/>
-    <col min="20" max="20" width="10" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="10" max="10" width="19" customWidth="1"/>
+    <col min="11" max="12" width="26" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="26" customWidth="1"/>
+    <col min="15" max="15" width="12" customWidth="1"/>
+    <col min="16" max="16" width="13" customWidth="1"/>
+    <col min="17" max="19" width="12" customWidth="1"/>
+    <col min="20" max="20" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -748,13 +757,75 @@
         <v>49</v>
       </c>
       <c r="R3" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="S3" t="s">
         <v>34</v>
       </c>
       <c r="T3" t="s">
-        <v>35</v>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" t="s">
+        <v>55</v>
+      </c>
+      <c r="G4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J4" t="s">
+        <v>48</v>
+      </c>
+      <c r="K4" t="s">
+        <v>48</v>
+      </c>
+      <c r="L4" t="s">
+        <v>48</v>
+      </c>
+      <c r="M4" t="s">
+        <v>48</v>
+      </c>
+      <c r="N4" t="s">
+        <v>48</v>
+      </c>
+      <c r="O4" t="s">
+        <v>48</v>
+      </c>
+      <c r="P4" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>48</v>
+      </c>
+      <c r="R4" t="s">
+        <v>48</v>
+      </c>
+      <c r="S4" t="s">
+        <v>48</v>
+      </c>
+      <c r="T4" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: complete import features for empresas and clientes-contabilidade (epic 11)
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/medicos-modelo.xlsx
+++ b/apps/web/public/templates/medicos-modelo.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Medicos" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Médicos" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="77">
   <si>
     <t>cpf</t>
   </si>
@@ -49,6 +49,9 @@
     <t>email</t>
   </si>
   <si>
+    <t>whatsapp</t>
+  </si>
+  <si>
     <t>cep</t>
   </si>
   <si>
@@ -73,6 +76,45 @@
     <t>conta_emissora</t>
   </si>
   <si>
+    <t>modo_cobranca</t>
+  </si>
+  <si>
+    <t>percentual_producao</t>
+  </si>
+  <si>
+    <t>dias_vencimento</t>
+  </si>
+  <si>
+    <t>multa_percent</t>
+  </si>
+  <si>
+    <t>juros_mes_percent</t>
+  </si>
+  <si>
+    <t>desconto_percent</t>
+  </si>
+  <si>
+    <t>desconto_dias</t>
+  </si>
+  <si>
+    <t>regra_preco_forma</t>
+  </si>
+  <si>
+    <t>regra_preco_base</t>
+  </si>
+  <si>
+    <t>regra_preco_limiar</t>
+  </si>
+  <si>
+    <t>regra_preco_taxa</t>
+  </si>
+  <si>
+    <t>regra_preco_valor_fixo</t>
+  </si>
+  <si>
+    <t>empresa_grupo</t>
+  </si>
+  <si>
     <t>12345678900</t>
   </si>
   <si>
@@ -97,6 +139,9 @@
     <t>fulano@exemplo.com</t>
   </si>
   <si>
+    <t>85999998888</t>
+  </si>
+  <si>
     <t>60000000</t>
   </si>
   <si>
@@ -121,6 +166,9 @@
     <t>mc</t>
   </si>
   <si>
+    <t>faixa_guias</t>
+  </si>
+  <si>
     <t>98765432100</t>
   </si>
   <si>
@@ -148,6 +196,9 @@
     <t>contato@ciclana.com</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>60110000</t>
   </si>
   <si>
@@ -157,9 +208,6 @@
     <t>2000</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Meireles</t>
   </si>
   <si>
@@ -179,6 +227,21 @@
   </si>
   <si>
     <t>sim</t>
+  </si>
+  <si>
+    <t>55566677788</t>
+  </si>
+  <si>
+    <t>Dr. Preco Proprio</t>
+  </si>
+  <si>
+    <t>Neurologia</t>
+  </si>
+  <si>
+    <t>preco_proprio</t>
+  </si>
+  <si>
+    <t>por_guia</t>
   </si>
 </sst>
 </file>
@@ -195,14 +258,20 @@
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F2937"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -219,7 +288,9 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -559,28 +630,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:AH5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="7" width="19" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="7" width="20" customWidth="1"/>
     <col min="8" max="8" width="25" customWidth="1"/>
-    <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="19" customWidth="1"/>
-    <col min="11" max="12" width="26" customWidth="1"/>
-    <col min="13" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="26" customWidth="1"/>
-    <col min="15" max="15" width="12" customWidth="1"/>
-    <col min="16" max="16" width="13" customWidth="1"/>
-    <col min="17" max="19" width="12" customWidth="1"/>
-    <col min="20" max="20" width="16" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="11" max="12" width="30" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="14" max="14" width="15" customWidth="1"/>
+    <col min="15" max="15" width="30" customWidth="1"/>
+    <col min="16" max="16" width="10" customWidth="1"/>
+    <col min="17" max="19" width="20" customWidth="1"/>
+    <col min="20" max="20" width="10" customWidth="1"/>
+    <col min="21" max="21" width="18" customWidth="1"/>
+    <col min="22" max="22" width="20" customWidth="1"/>
+    <col min="23" max="23" width="18" customWidth="1"/>
+    <col min="24" max="24" width="16" customWidth="1"/>
+    <col min="25" max="25" width="15" customWidth="1"/>
+    <col min="26" max="27" width="16" customWidth="1"/>
+    <col min="28" max="28" width="14" customWidth="1"/>
+    <col min="29" max="29" width="18" customWidth="1"/>
+    <col min="30" max="32" width="16" customWidth="1"/>
+    <col min="33" max="33" width="18" customWidth="1"/>
+    <col min="34" max="34" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="25" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -641,191 +720,250 @@
       <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J2" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L2" t="s">
+        <v>41</v>
+      </c>
+      <c r="M2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N2" t="s">
+        <v>43</v>
+      </c>
+      <c r="O2" t="s">
+        <v>44</v>
+      </c>
+      <c r="P2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>46</v>
+      </c>
+      <c r="R2" t="s">
+        <v>47</v>
+      </c>
+      <c r="S2" t="s">
+        <v>48</v>
+      </c>
+      <c r="T2" t="s">
+        <v>49</v>
+      </c>
+      <c r="U2" t="s">
+        <v>50</v>
+      </c>
+      <c r="V2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G3" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" t="s">
+        <v>56</v>
+      </c>
+      <c r="I3" t="s">
+        <v>57</v>
+      </c>
+      <c r="J3" t="s">
+        <v>58</v>
+      </c>
+      <c r="K3" t="s">
+        <v>59</v>
+      </c>
+      <c r="L3" t="s">
+        <v>60</v>
+      </c>
+      <c r="M3" t="s">
+        <v>61</v>
+      </c>
+      <c r="N3" t="s">
+        <v>62</v>
+      </c>
+      <c r="O3" t="s">
+        <v>63</v>
+      </c>
+      <c r="P3" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>61</v>
+      </c>
+      <c r="R3" t="s">
+        <v>65</v>
+      </c>
+      <c r="S3" t="s">
+        <v>48</v>
+      </c>
+      <c r="T3" t="s">
+        <v>49</v>
+      </c>
+      <c r="U3" t="s">
+        <v>66</v>
+      </c>
+      <c r="V3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F4" t="s">
+        <v>71</v>
+      </c>
+      <c r="G4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" t="s">
+        <v>39</v>
+      </c>
+      <c r="V4" t="s">
         <v>22</v>
       </c>
-      <c r="D2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F2" t="s">
-        <v>24</v>
-      </c>
-      <c r="G2" t="s">
-        <v>24</v>
-      </c>
-      <c r="H2" t="s">
-        <v>25</v>
-      </c>
-      <c r="I2" t="s">
-        <v>26</v>
-      </c>
-      <c r="J2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N2" t="s">
-        <v>29</v>
-      </c>
-      <c r="O2" t="s">
-        <v>30</v>
-      </c>
-      <c r="P2" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>32</v>
-      </c>
-      <c r="R2" t="s">
-        <v>33</v>
-      </c>
-      <c r="S2" t="s">
-        <v>34</v>
-      </c>
-      <c r="T2" t="s">
+      <c r="W4">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" t="s">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" t="s">
         <v>37</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E5" t="s">
         <v>38</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" t="s">
         <v>39</v>
       </c>
-      <c r="E3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H3" t="s">
-        <v>40</v>
-      </c>
-      <c r="I3" t="s">
-        <v>41</v>
-      </c>
-      <c r="J3" t="s">
-        <v>42</v>
-      </c>
-      <c r="K3" t="s">
-        <v>43</v>
-      </c>
-      <c r="L3" t="s">
-        <v>44</v>
-      </c>
-      <c r="M3" t="s">
-        <v>45</v>
-      </c>
-      <c r="N3" t="s">
-        <v>46</v>
-      </c>
-      <c r="O3" t="s">
-        <v>47</v>
-      </c>
-      <c r="P3" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>49</v>
-      </c>
-      <c r="R3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S3" t="s">
-        <v>34</v>
-      </c>
-      <c r="T3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E4" t="s">
-        <v>55</v>
-      </c>
-      <c r="F4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H4" t="s">
-        <v>25</v>
-      </c>
-      <c r="I4" t="s">
-        <v>48</v>
-      </c>
-      <c r="J4" t="s">
-        <v>48</v>
-      </c>
-      <c r="K4" t="s">
-        <v>48</v>
-      </c>
-      <c r="L4" t="s">
-        <v>48</v>
-      </c>
-      <c r="M4" t="s">
-        <v>48</v>
-      </c>
-      <c r="N4" t="s">
-        <v>48</v>
-      </c>
-      <c r="O4" t="s">
-        <v>48</v>
-      </c>
-      <c r="P4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>48</v>
-      </c>
-      <c r="R4" t="s">
-        <v>48</v>
-      </c>
-      <c r="S4" t="s">
-        <v>48</v>
-      </c>
-      <c r="T4" t="s">
-        <v>48</v>
+      <c r="V5" t="s">
+        <v>75</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>76</v>
+      </c>
+      <c r="AF5">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>